<commit_message>
Update NY gaming data - Fri Oct 16 15:01:00 UTC 2026
</commit_message>
<xml_diff>
--- a/NY_State_Reports_2026-10-16/Bally_Bet_Weekly_Report.xlsx
+++ b/NY_State_Reports_2026-10-16/Bally_Bet_Weekly_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\MOBILE SPORTS WAGERING\11_Weekly Web Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EEA424E-1B7A-461D-85E0-C1184CAECC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EBD38A-7D57-43F4-BBA8-D6E59EDC1D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EDA5EF8F-B63B-4D9E-966F-AB4A019BBE74}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EDA5EF8F-B63B-4D9E-966F-AB4A019BBE74}"/>
   </bookViews>
   <sheets>
     <sheet name="FY 26-27" sheetId="6" r:id="rId1"/>
@@ -2816,7 +2816,12 @@
         <v>46306</v>
       </c>
       <c r="B41" s="20"/>
-      <c r="F41" s="23"/>
+      <c r="C41" s="21">
+        <v>3181152.45</v>
+      </c>
+      <c r="F41" s="23">
+        <v>336852.25999999995</v>
+      </c>
       <c r="G41"/>
       <c r="H41"/>
       <c r="I41"/>
@@ -3358,11 +3363,11 @@
       </c>
       <c r="C67" s="24">
         <f>SUM(C13:C66)</f>
-        <v>84950935.570000008</v>
+        <v>88132088.020000011</v>
       </c>
       <c r="F67" s="24">
         <f>SUM(F13:F66)</f>
-        <v>7535363.6700000009</v>
+        <v>7872215.9300000006</v>
       </c>
       <c r="G67"/>
       <c r="H67"/>

</xml_diff>